<commit_message>
feat: add extended operational fields for SharePoint and Master Admin recovery flow
</commit_message>
<xml_diff>
--- a/AppDB.xlsx
+++ b/AppDB.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="Rbadf144ca52e4bd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headcount" sheetId="2" r:id="R7d0ac449af314075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faltas" sheetId="3" r:id="R189a969237d54c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kudos" sheetId="4" r:id="Rb8bf44564a4544b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocupacion" sheetId="5" r:id="Re050cfbc7cb8411e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="R14ca88fa7a4140be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headcount" sheetId="2" r:id="R50c068bc5077463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faltas" sheetId="3" r:id="R551f317fce194ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kudos" sheetId="4" r:id="Re8d718dd91f44c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocupacion" sheetId="5" r:id="R4e71cb48308a46f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notificaciones" sheetId="6" r:id="R12271d7bf01b491d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,8 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -86,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -167,6 +169,9 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -211,8 +216,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabla_Headcount" displayName="Tabla_Headcount" ref="A1:G1" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G1"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabla_Headcount" displayName="Tabla_Headcount" ref="A1:G2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G2"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="EmailEmpleado"/>
@@ -227,9 +232,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabla_Faltas" displayName="Tabla_Faltas" ref="A1:K1" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:K1"/>
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabla_Faltas" displayName="Tabla_Faltas" ref="A1:T2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:T2"/>
+  <x:tableColumns count="20">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="EmailEmpleado"/>
     <x:tableColumn id="3" name="NombreEmpleado"/>
@@ -241,14 +246,23 @@
     <x:tableColumn id="9" name="RequiereAmonestacion"/>
     <x:tableColumn id="10" name="Sincronizado"/>
     <x:tableColumn id="11" name="FechaCreacion"/>
+    <x:tableColumn id="12" name="IdCasoHelpdesk"/>
+    <x:tableColumn id="13" name="ProcesoArea"/>
+    <x:tableColumn id="14" name="HorasPerdidas"/>
+    <x:tableColumn id="15" name="MinutosTardanza"/>
+    <x:tableColumn id="16" name="HoraLlegada"/>
+    <x:tableColumn id="17" name="OrigenError"/>
+    <x:tableColumn id="18" name="SubcategoriaError"/>
+    <x:tableColumn id="19" name="ComentariosCapacitacion"/>
+    <x:tableColumn id="20" name="IdAuditoria"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tabla_Kudos" displayName="Tabla_Kudos" ref="A1:H1" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H1"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tabla_Kudos" displayName="Tabla_Kudos" ref="A1:H2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H2"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="EmailEmisor"/>
@@ -264,8 +278,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Tabla_Ocupacion" displayName="Tabla_Ocupacion" ref="A1:G1" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G1"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Tabla_Ocupacion" displayName="Tabla_Ocupacion" ref="A1:G2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G2"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="EmailEmpleado"/>
@@ -274,6 +288,21 @@
     <x:tableColumn id="5" name="CoberturaAsignada"/>
     <x:tableColumn id="6" name="Observaciones"/>
     <x:tableColumn id="7" name="Sincronizado"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Tabla_Notificaciones" displayName="Tabla_Notificaciones" ref="A1:F2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F2"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="ID"/>
+    <x:tableColumn id="2" name="Tipo"/>
+    <x:tableColumn id="3" name="Destinatario"/>
+    <x:tableColumn id="4" name="Mensaje"/>
+    <x:tableColumn id="5" name="Fecha"/>
+    <x:tableColumn id="6" name="Sincronizado"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -535,16 +564,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H2" s="22" t="n">
-        <x:v>46237.14325231482</x:v>
+        <x:v>46237.24369231481</x:v>
       </x:c>
       <x:c r="I2" s="22" t="n">
-        <x:v>46237.14325231482</x:v>
+        <x:v>46237.24369231481</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c4b8c09ae4847a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0502a4e3804141ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -585,10 +614,19 @@
         <x:v>EstadoActivo</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ac6201700e1435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04c1622264e7495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -608,6 +646,15 @@
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="26" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="30" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="42" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -641,14 +688,63 @@
       <x:c r="J1" s="13" t="str">
         <x:v>Sincronizado</x:v>
       </x:c>
-      <x:c r="K1" s="14" t="str">
+      <x:c r="K1" s="13" t="str">
         <x:v>FechaCreacion</x:v>
       </x:c>
+      <x:c r="L1" s="13" t="str">
+        <x:v>IdCasoHelpdesk</x:v>
+      </x:c>
+      <x:c r="M1" s="13" t="str">
+        <x:v>ProcesoArea</x:v>
+      </x:c>
+      <x:c r="N1" s="13" t="str">
+        <x:v>HorasPerdidas</x:v>
+      </x:c>
+      <x:c r="O1" s="13" t="str">
+        <x:v>MinutosTardanza</x:v>
+      </x:c>
+      <x:c r="P1" s="13" t="str">
+        <x:v>HoraLlegada</x:v>
+      </x:c>
+      <x:c r="Q1" s="13" t="str">
+        <x:v>OrigenError</x:v>
+      </x:c>
+      <x:c r="R1" s="13" t="str">
+        <x:v>SubcategoriaError</x:v>
+      </x:c>
+      <x:c r="S1" s="13" t="str">
+        <x:v>ComentariosCapacitacion</x:v>
+      </x:c>
+      <x:c r="T1" s="14" t="str">
+        <x:v>IdAuditoria</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+      <x:c r="H2" s="20"/>
+      <x:c r="I2" s="20"/>
+      <x:c r="J2" s="20"/>
+      <x:c r="K2" s="20"/>
+      <x:c r="L2" s="20"/>
+      <x:c r="M2" s="20"/>
+      <x:c r="N2" s="24"/>
+      <x:c r="O2" s="24"/>
+      <x:c r="P2" s="20"/>
+      <x:c r="Q2" s="20"/>
+      <x:c r="R2" s="20"/>
+      <x:c r="S2" s="20"/>
+      <x:c r="T2" s="20"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc04a7b01d7ea41b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf16eaf630e14932"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -693,10 +789,20 @@
         <x:v>Sincronizado</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+      <x:c r="H2" s="20"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5f63edaac00404c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04468bea97604a1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -737,10 +843,67 @@
         <x:v>Sincronizado</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R460302f530804542"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0682b154730b4c9b"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="12" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Tipo</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Destinatario</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Mensaje</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Fecha</x:v>
+      </x:c>
+      <x:c r="F1" s="14" t="str">
+        <x:v>Sincronizado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="20"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27c69dfb393f42d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>